<commit_message>
codegen: complete Luban SourceGenerator core pipeline
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.ability.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.ability.xlsx
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.33203125" customWidth="1" style="8" min="4" max="5"/>
@@ -821,67 +821,49 @@
     <row r="4">
       <c r="A4" s="9" t="n"/>
       <c r="B4" s="9" t="n">
-        <v>10001</v>
+        <v>10002</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>move</t>
+          <t>RunSpeedUp</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>移动</t>
+          <t>加速</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
       <c r="F4" s="9" t="inlineStr"/>
       <c r="G4" s="9" t="inlineStr"/>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>2002</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>3001</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>0;0;2010</t>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>3001;0;0</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>MoveInput</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>0.5</v>
+          <t>ApplyEffectsOnActivate</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1002;1001</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="9" t="n">
-        <v>10002</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>RunSpeedUp</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>加速</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="9" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>3001;0;0</t>
+      <c r="B5" t="n">
+        <v>1003</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>debug_ge_ability</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>调试GE</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -891,22 +873,22 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>1002;1001</t>
+          <t>1003</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="n">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>debug_ge_ability</t>
+          <t>debug_ge_2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>调试GE</t>
+          <t>调试ge2</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -916,116 +898,91 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1005</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="n">
-        <v>1005</v>
+        <v>20001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>debug_ge_2</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>调试ge2</t>
+          <t>玩家普通攻击</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>3003</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0;0;3003</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>ApplyEffectsOnActivate</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>1005</t>
-        </is>
+          <t>TimelineRef</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="n">
-        <v>20001</v>
+        <v>5000</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Attack</t>
+          <t>Dodge</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
-        <is>
-          <t>玩家普通攻击</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>3003</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>0;0;3003</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>TimelineRef</t>
-        </is>
-      </c>
-      <c r="O8" t="n">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Dodge</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">闪避
 </t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E8" t="n">
         <v>3002</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F8" t="n">
         <v>3001</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G8" t="n">
         <v>120</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>3003;0;0</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="K8" t="n">
         <v>3002</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>0;0;3002</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>TimelineRef</t>
         </is>
       </c>
-      <c r="O9" t="n">
+      <c r="O8" t="n">
         <v>103</v>
       </c>
     </row>

</xml_diff>

<commit_message>
codegen: add generated ability commit gate
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.ability.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.ability.xlsx
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.33203125" customWidth="1" style="8" min="4" max="5"/>
@@ -986,6 +986,81 @@
         <v>103</v>
       </c>
     </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>9101</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AutoChessPlayerAttack</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>AutoChess player attack ability</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>ApplyEffectsOnActivate</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>9201</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="n">
+        <v>9102</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AutoChessEnemyAttack</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AutoChess enemy attack ability</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>ApplyEffectsOnActivate</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>9202</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="n">
+        <v>9103</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AutoChessPlayerExecute</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AutoChess player execute ability</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ApplyEffectsOnActivate</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>9207</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="N1:AA1"/>

</xml_diff>